<commit_message>
Import the 10-02 export and record what the new format did
Five films now carry the current rules. Reading load fell 36% (21.9 to 14.1 characters/second) and the average watch time did not move: 7.17s against 7.31s for the September films. Completion halved, which is arithmetic — the denominator went from 12 seconds to 21 — and completion against plays is +0.048, so it is not the metric to protect.

What the data does say: viewers leave at about seven seconds whatever the film's length, so the extra nine seconds bought nothing; and the spread inside the new format (2s bounce 20.9% to 43.0%) is wider than the gap between formats, which puts the lever at the opening rather than in the layout.
</commit_message>
<xml_diff>
--- a/dataExport/作品列表导出.xlsx
+++ b/dataExport/作品列表导出.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="422">
   <si>
     <t>作品名称</t>
   </si>
@@ -64,6 +64,162 @@
   </si>
   <si>
     <t>粉丝增量</t>
+  </si>
+  <si>
+    <t>决明子：又名草决明 《神农本草经》卷一·上经载决明子。
+  本片照录原文，逐句今译，并说明「青盲」「白膜」在汉代指什么。
+  古籍内容展示，不构成诊疗建议。
+#神农本草经  #本草  #古籍  #传统文化  #读书</t>
+  </si>
+  <si>
+    <t>2026-10-01 19:00:00</t>
+  </si>
+  <si>
+    <t>1min-视频</t>
+  </si>
+  <si>
+    <t>公开</t>
+  </si>
+  <si>
+    <t>1148</t>
+  </si>
+  <si>
+    <t>0.112142</t>
+  </si>
+  <si>
+    <t>0.399072</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>0.235112</t>
+  </si>
+  <si>
+    <t>10.778036</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>防风：古书说的「大风」是什么 《神农本草经》卷一·上经载防风。
+  本片照录原文，逐句今译，并说明「大风」「痹」在汉代指什么。
+  古籍内容展示，不构成诊疗建议。
+#神农本草经  #本草  #古籍  #传统文化  #读书</t>
+  </si>
+  <si>
+    <t>2026-10-01 08:00:00</t>
+  </si>
+  <si>
+    <t>689</t>
+  </si>
+  <si>
+    <t>0.044140</t>
+  </si>
+  <si>
+    <t>0.241679</t>
+  </si>
+  <si>
+    <t>0.429812</t>
+  </si>
+  <si>
+    <t>5.342981</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>蓝实：古书里的染青草 《神农本草经》卷一·上经载蓝实。
+  本片照录原文，逐句今译，并说明「蛊」「注鬼」是汉代的病名观念。
+  古籍内容展示，不构成诊疗建议。
+#神农本草经  #本草  #古籍  #传统文化  #读书</t>
+  </si>
+  <si>
+    <t>2026-09-30 19:00:00</t>
+  </si>
+  <si>
+    <t>708</t>
+  </si>
+  <si>
+    <t>0.092414</t>
+  </si>
+  <si>
+    <t>0.283444</t>
+  </si>
+  <si>
+    <t>0.324503</t>
+  </si>
+  <si>
+    <t>6.480795</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>紫芝：六芝之一，色紫如桑 《神农本草经》卷一·上经载紫芝。
+  本片照录原文，逐句今译，并说明「保神」「好颜色」在汉代是什么意思。
+  古籍内容展示，不构成诊疗建议。
+#神农本草经  #本草  #古籍古书  #传统文化  #读书</t>
+  </si>
+  <si>
+    <t>2026-09-30 08:00:00</t>
+  </si>
+  <si>
+    <t>1863</t>
+  </si>
+  <si>
+    <t>0.062771</t>
+  </si>
+  <si>
+    <t>0.343880</t>
+  </si>
+  <si>
+    <t>0.241183</t>
+  </si>
+  <si>
+    <t>7.210062</t>
+  </si>
+  <si>
+    <t>黄芝：古书说它黄如紫金 《神农本草经》卷一·上经载黄芝。
+本片照录原文，逐句今译，附注释说明，并配灵芝照片（Ganoderma curtisii）。
+古籍内容展示，不构成诊疗建议。
+#黄芝  #神农本草经  #中医  #中草药 #中药材</t>
+  </si>
+  <si>
+    <t>2026-09-27 19:19:09</t>
+  </si>
+  <si>
+    <t>1667</t>
+  </si>
+  <si>
+    <t>0.067463</t>
+  </si>
+  <si>
+    <t>0.323569</t>
+  </si>
+  <si>
+    <t>0.209128</t>
+  </si>
+  <si>
+    <t>6.051090</t>
   </si>
   <si>
     <t>白芝：入肺应秋的玉芝 《神农本草经》卷一上经的白芝：味辛平，主咳逆上气、益肺气、通利口鼻、安魄。
@@ -75,43 +231,28 @@
     <t>2026-09-25 08:00:00</t>
   </si>
   <si>
-    <t>1min-视频</t>
-  </si>
-  <si>
-    <t>公开</t>
-  </si>
-  <si>
-    <t>1944</t>
-  </si>
-  <si>
-    <t>0.139808</t>
-  </si>
-  <si>
-    <t>0.345390</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>0.270504</t>
-  </si>
-  <si>
-    <t>6.700458</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>0</t>
+    <t>1961</t>
+  </si>
+  <si>
+    <t>0.140010</t>
+  </si>
+  <si>
+    <t>0.343812</t>
+  </si>
+  <si>
+    <t>0.273453</t>
+  </si>
+  <si>
+    <t>6.667665</t>
+  </si>
+  <si>
+    <t>19</t>
   </si>
   <si>
     <t>12</t>
   </si>
   <si>
     <t>11</t>
-  </si>
-  <si>
-    <t>6</t>
   </si>
   <si>
     <t>青芝：入肝应春的明目芝 《神农本草经》卷一上经的青芝：味酸平，主明目、补肝气、安精魂。
@@ -123,34 +264,22 @@
     <t>2026-09-24 19:00:00</t>
   </si>
   <si>
-    <t>1077</t>
-  </si>
-  <si>
-    <t>0.127014</t>
-  </si>
-  <si>
-    <t>0.298043</t>
-  </si>
-  <si>
-    <t>0.320285</t>
-  </si>
-  <si>
-    <t>6.495552</t>
+    <t>1092</t>
+  </si>
+  <si>
+    <t>0.125693</t>
+  </si>
+  <si>
+    <t>0.294271</t>
+  </si>
+  <si>
+    <t>0.317708</t>
+  </si>
+  <si>
+    <t>6.446181</t>
   </si>
   <si>
     <t>13</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>4</t>
   </si>
   <si>
     <t>赤芝：六芝之首的安神上品 《神农本草经》卷一上经的赤芝：味苦平，益心气、补中、增智慧、不忘。
@@ -162,19 +291,19 @@
     <t>2026-09-24 08:00:00</t>
   </si>
   <si>
-    <t>2950</t>
-  </si>
-  <si>
-    <t>0.111416</t>
-  </si>
-  <si>
-    <t>0.307897</t>
-  </si>
-  <si>
-    <t>0.284531</t>
-  </si>
-  <si>
-    <t>5.902100</t>
+    <t>2961</t>
+  </si>
+  <si>
+    <t>0.113001</t>
+  </si>
+  <si>
+    <t>0.309293</t>
+  </si>
+  <si>
+    <t>0.283788</t>
+  </si>
+  <si>
+    <t>5.912049</t>
   </si>
   <si>
     <t>10</t>
@@ -192,19 +321,22 @@
     <t>2026-09-23 20:00:00</t>
   </si>
   <si>
-    <t>1074</t>
-  </si>
-  <si>
-    <t>0.183511</t>
-  </si>
-  <si>
-    <t>0.421227</t>
-  </si>
-  <si>
-    <t>0.228027</t>
-  </si>
-  <si>
-    <t>6.970149</t>
+    <t>1081</t>
+  </si>
+  <si>
+    <t>0.188215</t>
+  </si>
+  <si>
+    <t>0.422824</t>
+  </si>
+  <si>
+    <t>0.226601</t>
+  </si>
+  <si>
+    <t>6.987685</t>
+  </si>
+  <si>
+    <t>8</t>
   </si>
   <si>
     <t>奄闾子：食之神仙的蒿类 《神农本草经》卷一上经的奄闾子：味苦微寒，主五脏瘀血、腹中水气、身体诸痛。
@@ -216,22 +348,19 @@
     <t>2026-09-23 08:00:00</t>
   </si>
   <si>
-    <t>783</t>
-  </si>
-  <si>
-    <t>0.176556</t>
-  </si>
-  <si>
-    <t>0.440655</t>
-  </si>
-  <si>
-    <t>0.251023</t>
-  </si>
-  <si>
-    <t>8.118690</t>
-  </si>
-  <si>
-    <t>3</t>
+    <t>793</t>
+  </si>
+  <si>
+    <t>0.174037</t>
+  </si>
+  <si>
+    <t>0.433962</t>
+  </si>
+  <si>
+    <t>0.253369</t>
+  </si>
+  <si>
+    <t>8.045760</t>
   </si>
   <si>
     <t>析子：俗呼老荠的明目药 《神农本草经》卷一上经的析子（菥蓂）：味辛微温，主目痛泪出、益精光。
@@ -243,25 +372,19 @@
     <t>2026-09-22 20:00:00</t>
   </si>
   <si>
-    <t>664</t>
-  </si>
-  <si>
-    <t>0.148611</t>
-  </si>
-  <si>
-    <t>0.370565</t>
-  </si>
-  <si>
-    <t>0.252300</t>
-  </si>
-  <si>
-    <t>8.708279</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>667</t>
+  </si>
+  <si>
+    <t>0.147994</t>
+  </si>
+  <si>
+    <t>0.370904</t>
+  </si>
+  <si>
+    <t>0.251638</t>
+  </si>
+  <si>
+    <t>8.705111</t>
   </si>
   <si>
     <t>赤箭：其实就是天麻 《神农本草经》卷一上经的赤箭：味辛温，主杀鬼精物蛊毒恶气，久服增年。
@@ -273,22 +396,19 @@
     <t>2026-09-22 08:00:00</t>
   </si>
   <si>
-    <t>1899</t>
-  </si>
-  <si>
-    <t>0.152000</t>
-  </si>
-  <si>
-    <t>0.377130</t>
-  </si>
-  <si>
-    <t>0.220628</t>
-  </si>
-  <si>
-    <t>8.162332</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>1902</t>
+  </si>
+  <si>
+    <t>0.151572</t>
+  </si>
+  <si>
+    <t>0.376118</t>
+  </si>
+  <si>
+    <t>0.220930</t>
+  </si>
+  <si>
+    <t>8.146691</t>
   </si>
   <si>
     <t>白蒿：《诗经》里的采蘩 《神农本草经》卷一上经的白蒿：味甘平，补中益气，长毛发令黑，疗心悬。
@@ -300,19 +420,19 @@
     <t>2026-09-21 19:00:00</t>
   </si>
   <si>
-    <t>1964</t>
-  </si>
-  <si>
-    <t>0.120995</t>
-  </si>
-  <si>
-    <t>0.331504</t>
-  </si>
-  <si>
-    <t>0.256516</t>
-  </si>
-  <si>
-    <t>5.891175</t>
+    <t>1968</t>
+  </si>
+  <si>
+    <t>0.120821</t>
+  </si>
+  <si>
+    <t>0.331050</t>
+  </si>
+  <si>
+    <t>0.256164</t>
+  </si>
+  <si>
+    <t>5.887215</t>
   </si>
   <si>
     <t>14</t>
@@ -327,19 +447,19 @@
     <t>2026-09-21 08:00:00</t>
   </si>
   <si>
-    <t>2945</t>
-  </si>
-  <si>
-    <t>0.164363</t>
-  </si>
-  <si>
-    <t>0.383844</t>
-  </si>
-  <si>
-    <t>0.240905</t>
-  </si>
-  <si>
-    <t>8.939559</t>
+    <t>2948</t>
+  </si>
+  <si>
+    <t>0.164314</t>
+  </si>
+  <si>
+    <t>0.384197</t>
+  </si>
+  <si>
+    <t>0.240767</t>
+  </si>
+  <si>
+    <t>8.964787</t>
   </si>
   <si>
     <t>17</t>
@@ -354,19 +474,19 @@
     <t>2026-09-20 19:00:00</t>
   </si>
   <si>
-    <t>3016</t>
-  </si>
-  <si>
-    <t>0.188143</t>
-  </si>
-  <si>
-    <t>0.426230</t>
-  </si>
-  <si>
-    <t>0.223019</t>
-  </si>
-  <si>
-    <t>7.623634</t>
+    <t>3018</t>
+  </si>
+  <si>
+    <t>0.188077</t>
+  </si>
+  <si>
+    <t>0.426425</t>
+  </si>
+  <si>
+    <t>0.222943</t>
+  </si>
+  <si>
+    <t>7.624445</t>
   </si>
   <si>
     <t>20</t>
@@ -381,19 +501,19 @@
     <t>2026-09-20 14:08:36</t>
   </si>
   <si>
-    <t>583</t>
-  </si>
-  <si>
-    <t>0.152244</t>
-  </si>
-  <si>
-    <t>0.380090</t>
-  </si>
-  <si>
-    <t>0.251885</t>
-  </si>
-  <si>
-    <t>7.334842</t>
+    <t>585</t>
+  </si>
+  <si>
+    <t>0.152000</t>
+  </si>
+  <si>
+    <t>0.381024</t>
+  </si>
+  <si>
+    <t>0.251506</t>
+  </si>
+  <si>
+    <t>7.335843</t>
   </si>
   <si>
     <t>细辛：华阴色白者为善 《神农本草经》卷一上经的细辛：味辛温，主头痛脑动、百节拘挛、风湿痹痛。
@@ -405,19 +525,19 @@
     <t>2026-09-19 19:00:00</t>
   </si>
   <si>
-    <t>1374</t>
-  </si>
-  <si>
-    <t>0.108819</t>
-  </si>
-  <si>
-    <t>0.299046</t>
-  </si>
-  <si>
-    <t>0.353542</t>
-  </si>
-  <si>
-    <t>5.698910</t>
+    <t>1376</t>
+  </si>
+  <si>
+    <t>0.109453</t>
+  </si>
+  <si>
+    <t>0.299523</t>
+  </si>
+  <si>
+    <t>0.353302</t>
+  </si>
+  <si>
+    <t>5.703880</t>
   </si>
   <si>
     <t>龙胆：主骨间寒热的苦口上品 《神农本草经》卷一上经的龙胆：味苦涩，主惊痫邪气、续绝伤、杀蛊毒。
@@ -429,19 +549,22 @@
     <t>2026-09-19 08:00:00</t>
   </si>
   <si>
-    <t>2967</t>
-  </si>
-  <si>
-    <t>0.149035</t>
-  </si>
-  <si>
-    <t>0.364213</t>
-  </si>
-  <si>
-    <t>0.269670</t>
-  </si>
-  <si>
-    <t>7.196383</t>
+    <t>2977</t>
+  </si>
+  <si>
+    <t>0.149070</t>
+  </si>
+  <si>
+    <t>0.364557</t>
+  </si>
+  <si>
+    <t>0.269620</t>
+  </si>
+  <si>
+    <t>7.194304</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>远志：它的叶子叫小草 《神农本草经》卷一上经的远志：味苦温，利九窍、益智慧、不忘、强志倍力。
@@ -453,22 +576,19 @@
     <t>2026-09-18 19:00:00</t>
   </si>
   <si>
-    <t>1948</t>
-  </si>
-  <si>
-    <t>0.128244</t>
-  </si>
-  <si>
-    <t>0.306888</t>
-  </si>
-  <si>
-    <t>0.327791</t>
-  </si>
-  <si>
-    <t>6.136817</t>
-  </si>
-  <si>
-    <t>16</t>
+    <t>1959</t>
+  </si>
+  <si>
+    <t>0.127797</t>
+  </si>
+  <si>
+    <t>0.306818</t>
+  </si>
+  <si>
+    <t>0.329072</t>
+  </si>
+  <si>
+    <t>6.126894</t>
   </si>
   <si>
     <t>泽泻：能行水上的本经奇谈 《神农本草经》卷一上经的泽泻：味甘寒，主风寒湿痹、乳难，消水养五脏。
@@ -480,19 +600,19 @@
     <t>2026-09-18 08:00:00</t>
   </si>
   <si>
-    <t>2791</t>
-  </si>
-  <si>
-    <t>0.145999</t>
-  </si>
-  <si>
-    <t>0.364489</t>
-  </si>
-  <si>
-    <t>0.238500</t>
-  </si>
-  <si>
-    <t>7.506885</t>
+    <t>2800</t>
+  </si>
+  <si>
+    <t>0.145910</t>
+  </si>
+  <si>
+    <t>0.364275</t>
+  </si>
+  <si>
+    <t>0.238360</t>
+  </si>
+  <si>
+    <t>7.504246</t>
   </si>
   <si>
     <t>薏苡仁：马援常饵的轻身药 《神农本草经》卷一上经的薏苡仁：味甘微寒，主拘挛不可屈伸、风湿痹、下气。
@@ -504,19 +624,19 @@
     <t>2026-09-17 19:00:00</t>
   </si>
   <si>
-    <t>2453</t>
-  </si>
-  <si>
-    <t>0.143575</t>
-  </si>
-  <si>
-    <t>0.365188</t>
-  </si>
-  <si>
-    <t>0.267577</t>
-  </si>
-  <si>
-    <t>7.501024</t>
+    <t>2459</t>
+  </si>
+  <si>
+    <t>0.143318</t>
+  </si>
+  <si>
+    <t>0.365588</t>
+  </si>
+  <si>
+    <t>0.267462</t>
+  </si>
+  <si>
+    <t>7.499148</t>
   </si>
   <si>
     <t>署豫：就是后来的山药 《神农本草经》卷一上经的署豫（薯蓣）：味甘温，主伤中、补虚羸、益气力、长肌肉。
@@ -528,19 +648,19 @@
     <t>2026-09-17 08:00:00</t>
   </si>
   <si>
-    <t>2813</t>
-  </si>
-  <si>
-    <t>0.158406</t>
-  </si>
-  <si>
-    <t>0.400803</t>
-  </si>
-  <si>
-    <t>0.234858</t>
-  </si>
-  <si>
-    <t>7.385352</t>
+    <t>2814</t>
+  </si>
+  <si>
+    <t>0.158355</t>
+  </si>
+  <si>
+    <t>0.400989</t>
+  </si>
+  <si>
+    <t>0.234785</t>
+  </si>
+  <si>
+    <t>7.385542</t>
   </si>
   <si>
     <t>木香：辟毒疫温鬼的本经香药 《神农本草经》卷一上经的木香：味辛，主邪气、辟毒疫温鬼、强志。
@@ -552,19 +672,19 @@
     <t>2026-09-16 19:00:00</t>
   </si>
   <si>
-    <t>1310</t>
-  </si>
-  <si>
-    <t>0.119885</t>
-  </si>
-  <si>
-    <t>0.307208</t>
-  </si>
-  <si>
-    <t>0.247726</t>
-  </si>
-  <si>
-    <t>5.695591</t>
+    <t>1317</t>
+  </si>
+  <si>
+    <t>0.120344</t>
+  </si>
+  <si>
+    <t>0.307263</t>
+  </si>
+  <si>
+    <t>0.247905</t>
+  </si>
+  <si>
+    <t>5.699022</t>
   </si>
   <si>
     <t>车前子：牛迹里长出的当道草 《神农本草经》卷一上经的车前子：味甘寒，主气癃、利水道小便、除湿痹。
@@ -576,22 +696,25 @@
     <t>2026-09-16 08:00:00</t>
   </si>
   <si>
-    <t>4856</t>
-  </si>
-  <si>
-    <t>0.210498</t>
-  </si>
-  <si>
-    <t>0.458306</t>
-  </si>
-  <si>
-    <t>0.219980</t>
-  </si>
-  <si>
-    <t>10.194963</t>
+    <t>4862</t>
+  </si>
+  <si>
+    <t>0.210414</t>
+  </si>
+  <si>
+    <t>0.458104</t>
+  </si>
+  <si>
+    <t>0.220057</t>
+  </si>
+  <si>
+    <t>10.188739</t>
   </si>
   <si>
     <t>28</t>
+  </si>
+  <si>
+    <t>16</t>
   </si>
   <si>
     <t>独活：无风自动的本经上品 《神农本草经》卷一上经的独活：味苦平，主风寒所击、金疮止痛、女子疝瘕。
@@ -603,22 +726,19 @@
     <t>2026-09-15 20:06:14</t>
   </si>
   <si>
-    <t>2917</t>
-  </si>
-  <si>
-    <t>0.161770</t>
-  </si>
-  <si>
-    <t>0.371988</t>
-  </si>
-  <si>
-    <t>0.274012</t>
-  </si>
-  <si>
-    <t>8.176565</t>
-  </si>
-  <si>
-    <t>21</t>
+    <t>2921</t>
+  </si>
+  <si>
+    <t>0.161551</t>
+  </si>
+  <si>
+    <t>0.371713</t>
+  </si>
+  <si>
+    <t>0.274214</t>
+  </si>
+  <si>
+    <t>8.170513</t>
   </si>
   <si>
     <t>麦门冬：别名不死药的润肺上品 《神农本草经》卷一上经的麦门冬：味甘平，主心腹结气、胃络脉绝、羸瘦短气。
@@ -630,19 +750,19 @@
     <t>2026-09-14 08:00:00</t>
   </si>
   <si>
-    <t>961</t>
-  </si>
-  <si>
-    <t>0.159864</t>
-  </si>
-  <si>
-    <t>0.366062</t>
-  </si>
-  <si>
-    <t>0.303095</t>
-  </si>
-  <si>
-    <t>7.515475</t>
+    <t>964</t>
+  </si>
+  <si>
+    <t>0.160633</t>
+  </si>
+  <si>
+    <t>0.367412</t>
+  </si>
+  <si>
+    <t>0.302449</t>
+  </si>
+  <si>
+    <t>7.519702</t>
   </si>
   <si>
     <t>防葵：博物志说它与狼毒相似 《神农本草经》卷一上经的防葵：味辛寒，主疝瘕肠泄、膀胱热结、惊邪狂走。
@@ -654,19 +774,19 @@
     <t>2026-09-13 20:00:00</t>
   </si>
   <si>
-    <t>4268</t>
-  </si>
-  <si>
-    <t>0.159838</t>
-  </si>
-  <si>
-    <t>0.415551</t>
-  </si>
-  <si>
-    <t>0.190065</t>
-  </si>
-  <si>
-    <t>7.665011</t>
+    <t>4278</t>
+  </si>
+  <si>
+    <t>0.159919</t>
+  </si>
+  <si>
+    <t>0.415624</t>
+  </si>
+  <si>
+    <t>0.190117</t>
+  </si>
+  <si>
+    <t>7.664437</t>
   </si>
   <si>
     <t>女萎：就是后来的玉竹 《神农本草经》卷一上经的女萎：味甘平，主中风暴热、跌筋结肉，久服好颜色。
@@ -678,19 +798,19 @@
     <t>2026-09-13 08:00:00</t>
   </si>
   <si>
-    <t>3298</t>
-  </si>
-  <si>
-    <t>0.128972</t>
-  </si>
-  <si>
-    <t>0.401297</t>
-  </si>
-  <si>
-    <t>0.181582</t>
-  </si>
-  <si>
-    <t>7.182879</t>
+    <t>3304</t>
+  </si>
+  <si>
+    <t>0.128834</t>
+  </si>
+  <si>
+    <t>0.401658</t>
+  </si>
+  <si>
+    <t>0.181394</t>
+  </si>
+  <si>
+    <t>7.181653</t>
   </si>
   <si>
     <t>充蔚子：本经里的益母草子 《神农本草经》卷一上经的充蔚子（茺蔚子）：味辛微温，主明目益精、除水气，茎可作浴汤。
@@ -702,19 +822,19 @@
     <t>2026-09-12 19:13:39</t>
   </si>
   <si>
-    <t>758</t>
-  </si>
-  <si>
-    <t>0.147497</t>
-  </si>
-  <si>
-    <t>0.341902</t>
-  </si>
-  <si>
-    <t>0.314910</t>
-  </si>
-  <si>
-    <t>6.976864</t>
+    <t>761</t>
+  </si>
+  <si>
+    <t>0.148448</t>
+  </si>
+  <si>
+    <t>0.342308</t>
+  </si>
+  <si>
+    <t>0.314103</t>
+  </si>
+  <si>
+    <t>6.982051</t>
   </si>
   <si>
     <t>牛膝：陶弘景说它茎像牛膝 《神农本草经》卷一上经的牛膝：味苦酸，主寒湿痿痹、膝痛不可屈伸，逐血气。
@@ -726,19 +846,19 @@
     <t>2026-08-30 14:00:00</t>
   </si>
   <si>
-    <t>3255</t>
-  </si>
-  <si>
-    <t>0.190294</t>
-  </si>
-  <si>
-    <t>0.422197</t>
-  </si>
-  <si>
-    <t>0.236754</t>
-  </si>
-  <si>
-    <t>8.748745</t>
+    <t>3257</t>
+  </si>
+  <si>
+    <t>0.190182</t>
+  </si>
+  <si>
+    <t>0.422520</t>
+  </si>
+  <si>
+    <t>0.236622</t>
+  </si>
+  <si>
+    <t>8.748049</t>
   </si>
   <si>
     <t>菟丝子：本经续绝伤的上品 《神农本草经》卷一上经的菟丝子：味辛平，主续绝伤、益气力、肥健，汁去面皯。
@@ -750,19 +870,19 @@
     <t>2026-08-30 08:00:00</t>
   </si>
   <si>
-    <t>109</t>
-  </si>
-  <si>
-    <t>0.250000</t>
-  </si>
-  <si>
-    <t>0.423077</t>
-  </si>
-  <si>
-    <t>0.238462</t>
-  </si>
-  <si>
-    <t>7.230769</t>
+    <t>111</t>
+  </si>
+  <si>
+    <t>0.247706</t>
+  </si>
+  <si>
+    <t>0.427481</t>
+  </si>
+  <si>
+    <t>0.236641</t>
+  </si>
+  <si>
+    <t>7.236641</t>
   </si>
   <si>
     <t>术：本经里"长服山精"的上品 《神农本草经》卷一上经的术：味苦温，主风寒湿痹、死肌、痉、疸，止汗除热消食。
@@ -774,19 +894,19 @@
     <t>2026-08-29 14:00:00</t>
   </si>
   <si>
-    <t>2451</t>
-  </si>
-  <si>
-    <t>0.145455</t>
-  </si>
-  <si>
-    <t>0.356399</t>
-  </si>
-  <si>
-    <t>0.254092</t>
-  </si>
-  <si>
-    <t>9.842634</t>
+    <t>2453</t>
+  </si>
+  <si>
+    <t>0.145616</t>
+  </si>
+  <si>
+    <t>0.356241</t>
+  </si>
+  <si>
+    <t>0.254458</t>
+  </si>
+  <si>
+    <t>9.834695</t>
   </si>
   <si>
     <t>干地黄：本经"填骨髓"的第一补药 《神农本草经》卷一上经的干地黄：味甘寒，主折跌绝筋、逐血痹、填骨髓，生者尤良。
@@ -798,19 +918,19 @@
     <t>2026-08-29 08:00:00</t>
   </si>
   <si>
-    <t>71</t>
-  </si>
-  <si>
-    <t>0.265625</t>
-  </si>
-  <si>
-    <t>0.367089</t>
-  </si>
-  <si>
-    <t>0.316456</t>
-  </si>
-  <si>
-    <t>6.860759</t>
+    <t>73</t>
+  </si>
+  <si>
+    <t>0.276923</t>
+  </si>
+  <si>
+    <t>0.375000</t>
+  </si>
+  <si>
+    <t>0.312500</t>
+  </si>
+  <si>
+    <t>6.925000</t>
   </si>
   <si>
     <t>天门冬：抱朴子也记了它一堆别名 《神农本草经》卷一上经的天门冬：味苦平，主诸暴风湿偏痹，强骨髓，杀三虫。
@@ -822,19 +942,19 @@
     <t>2026-08-28 08:00:00</t>
   </si>
   <si>
-    <t>1858</t>
-  </si>
-  <si>
-    <t>0.143458</t>
-  </si>
-  <si>
-    <t>0.361097</t>
-  </si>
-  <si>
-    <t>0.284408</t>
-  </si>
-  <si>
-    <t>7.360872</t>
+    <t>1865</t>
+  </si>
+  <si>
+    <t>0.143832</t>
+  </si>
+  <si>
+    <t>0.361238</t>
+  </si>
+  <si>
+    <t>0.284627</t>
+  </si>
+  <si>
+    <t>7.365063</t>
   </si>
   <si>
     <t>鞠华：本经里"目欲脱"的菊花 《神农本草经》卷一上经的鞠华（菊花）：味苦平，主风、头眩肿痛、目欲脱、泪出，久服耐老延年。
@@ -846,19 +966,19 @@
     <t>2026-08-27 14:00:00</t>
   </si>
   <si>
-    <t>531</t>
-  </si>
-  <si>
-    <t>0.116487</t>
-  </si>
-  <si>
-    <t>0.300172</t>
-  </si>
-  <si>
-    <t>0.322470</t>
-  </si>
-  <si>
-    <t>5.720412</t>
+    <t>534</t>
+  </si>
+  <si>
+    <t>0.116071</t>
+  </si>
+  <si>
+    <t>0.302048</t>
+  </si>
+  <si>
+    <t>0.322526</t>
+  </si>
+  <si>
+    <t>5.721843</t>
   </si>
   <si>
     <t>菖蒲：通九窍、明耳目的本经上品 《神农本草经》卷一上经的菖蒲：味辛温，主风寒湿痹、咳逆上气，开心孔，通九窍，明耳目。
@@ -870,19 +990,19 @@
     <t>2026-08-27 08:00:00</t>
   </si>
   <si>
-    <t>319</t>
-  </si>
-  <si>
-    <t>0.142405</t>
-  </si>
-  <si>
-    <t>0.335244</t>
-  </si>
-  <si>
-    <t>0.355301</t>
-  </si>
-  <si>
-    <t>5.825215</t>
+    <t>320</t>
+  </si>
+  <si>
+    <t>0.141956</t>
+  </si>
+  <si>
+    <t>0.337143</t>
+  </si>
+  <si>
+    <t>0.354286</t>
+  </si>
+  <si>
+    <t>5.837143</t>
   </si>
   <si>
     <t>扁青：本经主折跌痈肿 《神农本草经》里的扁青：味甘平，主目痛、折跌、痈肿、金创不疗，利精神。
@@ -894,16 +1014,19 @@
     <t>2026-08-26 14:00:00</t>
   </si>
   <si>
-    <t>154</t>
-  </si>
-  <si>
-    <t>0.129032</t>
-  </si>
-  <si>
-    <t>0.380952</t>
-  </si>
-  <si>
-    <t>7.750000</t>
+    <t>156</t>
+  </si>
+  <si>
+    <t>0.127389</t>
+  </si>
+  <si>
+    <t>0.247059</t>
+  </si>
+  <si>
+    <t>0.382353</t>
+  </si>
+  <si>
+    <t>7.688235</t>
   </si>
   <si>
     <t>白青：可消而为铜的本经石药 《神农本草经》里的白青：味甘平，主明目、利九窍、耳聋，杀诸毒、三虫。
@@ -915,19 +1038,19 @@
     <t>2026-08-26 08:00:00</t>
   </si>
   <si>
-    <t>631</t>
-  </si>
-  <si>
-    <t>0.152695</t>
-  </si>
-  <si>
-    <t>0.350501</t>
-  </si>
-  <si>
-    <t>0.250358</t>
-  </si>
-  <si>
-    <t>11.092990</t>
+    <t>632</t>
+  </si>
+  <si>
+    <t>0.152466</t>
+  </si>
+  <si>
+    <t>0.350000</t>
+  </si>
+  <si>
+    <t>0.251429</t>
+  </si>
+  <si>
+    <t>11.078571</t>
   </si>
   <si>
     <t>紫石英：绝孕十年无子的本经说法 《神农本草经》里的紫石英：味甘温，主心腹咳逆，补不足，有女子风寒在子宫的古说。
@@ -939,19 +1062,19 @@
     <t>2026-08-23 20:35:00</t>
   </si>
   <si>
-    <t>4619</t>
-  </si>
-  <si>
-    <t>0.115978</t>
-  </si>
-  <si>
-    <t>0.355174</t>
-  </si>
-  <si>
-    <t>0.225729</t>
-  </si>
-  <si>
-    <t>7.089093</t>
+    <t>4621</t>
+  </si>
+  <si>
+    <t>0.115930</t>
+  </si>
+  <si>
+    <t>0.355032</t>
+  </si>
+  <si>
+    <t>0.226038</t>
+  </si>
+  <si>
+    <t>7.086861</t>
   </si>
   <si>
     <t>22</t>
@@ -966,19 +1089,19 @@
     <t>2026-08-23 18:32:24</t>
   </si>
   <si>
-    <t>3625</t>
-  </si>
-  <si>
-    <t>0.101251</t>
-  </si>
-  <si>
-    <t>0.332362</t>
-  </si>
-  <si>
-    <t>0.260933</t>
-  </si>
-  <si>
-    <t>5.686589</t>
+    <t>3629</t>
+  </si>
+  <si>
+    <t>0.101398</t>
+  </si>
+  <si>
+    <t>0.331879</t>
+  </si>
+  <si>
+    <t>0.260908</t>
+  </si>
+  <si>
+    <t>5.680628</t>
   </si>
   <si>
     <t>23</t>
@@ -993,19 +1116,19 @@
     <t>2026-08-22 14:50:00</t>
   </si>
   <si>
-    <t>1564</t>
-  </si>
-  <si>
-    <t>0.125837</t>
-  </si>
-  <si>
-    <t>0.397946</t>
-  </si>
-  <si>
-    <t>0.247754</t>
-  </si>
-  <si>
-    <t>7.596277</t>
+    <t>1567</t>
+  </si>
+  <si>
+    <t>0.126000</t>
+  </si>
+  <si>
+    <t>0.397953</t>
+  </si>
+  <si>
+    <t>0.247601</t>
+  </si>
+  <si>
+    <t>7.589891</t>
   </si>
   <si>
     <t>禹余粮：名字从大禹治水来 《神农本草经》里的禹余粮：味甘寒，主咳逆、寒热烦满、血闭症瘕。
@@ -1017,19 +1140,19 @@
     <t>2026-08-22 10:39:43</t>
   </si>
   <si>
-    <t>484</t>
-  </si>
-  <si>
-    <t>0.138568</t>
-  </si>
-  <si>
-    <t>0.327623</t>
-  </si>
-  <si>
-    <t>0.308351</t>
-  </si>
-  <si>
-    <t>5.884368</t>
+    <t>485</t>
+  </si>
+  <si>
+    <t>0.139908</t>
+  </si>
+  <si>
+    <t>0.326964</t>
+  </si>
+  <si>
+    <t>0.307856</t>
+  </si>
+  <si>
+    <t>5.878981</t>
   </si>
   <si>
     <t>曾青：铜之精的本经石药 《神农本草经》里的曾青：味酸小寒，主目痛止泪，破症坚积聚，久服轻身。
@@ -1041,19 +1164,19 @@
     <t>2026-08-21 20:00:00</t>
   </si>
   <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>0.084337</t>
-  </si>
-  <si>
-    <t>0.297619</t>
-  </si>
-  <si>
-    <t>0.404762</t>
-  </si>
-  <si>
-    <t>4.416667</t>
+    <t>84</t>
+  </si>
+  <si>
+    <t>0.083333</t>
+  </si>
+  <si>
+    <t>0.294118</t>
+  </si>
+  <si>
+    <t>0.400000</t>
+  </si>
+  <si>
+    <t>4.388235</t>
   </si>
   <si>
     <t>空青：能化铜铁铅锡作金 《神农本草经》里的空青：味甘寒，主眚盲耳聋，通血脉，养精神，能化铜铁铅锡作金。
@@ -1065,19 +1188,19 @@
     <t>2026-08-21 09:52:17</t>
   </si>
   <si>
-    <t>289</t>
-  </si>
-  <si>
-    <t>0.156667</t>
-  </si>
-  <si>
-    <t>0.348243</t>
-  </si>
-  <si>
-    <t>0.287540</t>
-  </si>
-  <si>
-    <t>6.888179</t>
+    <t>290</t>
+  </si>
+  <si>
+    <t>0.155629</t>
+  </si>
+  <si>
+    <t>0.346032</t>
+  </si>
+  <si>
+    <t>0.288889</t>
+  </si>
+  <si>
+    <t>6.857143</t>
   </si>
   <si>
     <t>滑石：利小便的本经石药 《神农本草经》里的滑石：味甘寒，主身热泄、女子乳难、癃闭，利小便，益精气。
@@ -1089,19 +1212,19 @@
     <t>2026-08-19 09:14:26</t>
   </si>
   <si>
-    <t>850</t>
-  </si>
-  <si>
-    <t>0.115385</t>
-  </si>
-  <si>
-    <t>0.281139</t>
-  </si>
-  <si>
-    <t>0.349941</t>
-  </si>
-  <si>
-    <t>5.513642</t>
+    <t>851</t>
+  </si>
+  <si>
+    <t>0.115099</t>
+  </si>
+  <si>
+    <t>0.281657</t>
+  </si>
+  <si>
+    <t>0.349112</t>
+  </si>
+  <si>
+    <t>5.514793</t>
   </si>
   <si>
     <t>24</t>
@@ -1116,19 +1239,19 @@
     <t>2026-08-18 20:00:00</t>
   </si>
   <si>
-    <t>126</t>
-  </si>
-  <si>
-    <t>0.114504</t>
-  </si>
-  <si>
-    <t>0.275362</t>
-  </si>
-  <si>
-    <t>0.304348</t>
-  </si>
-  <si>
-    <t>5.217391</t>
+    <t>129</t>
+  </si>
+  <si>
+    <t>0.119403</t>
+  </si>
+  <si>
+    <t>0.276596</t>
+  </si>
+  <si>
+    <t>0.297872</t>
+  </si>
+  <si>
+    <t>5.319149</t>
   </si>
   <si>
     <t>硝石：本经主五脏积热 《神农本草经》里的硝石：味苦寒，主五脏积热，涤去蓄结饮食，推陈致新。
@@ -1140,22 +1263,19 @@
     <t>2026-08-18 09:08:09</t>
   </si>
   <si>
-    <t>3254</t>
-  </si>
-  <si>
-    <t>0.135840</t>
-  </si>
-  <si>
-    <t>0.379654</t>
-  </si>
-  <si>
-    <t>0.235708</t>
-  </si>
-  <si>
-    <t>7.125183</t>
-  </si>
-  <si>
-    <t>19</t>
+    <t>3261</t>
+  </si>
+  <si>
+    <t>0.135716</t>
+  </si>
+  <si>
+    <t>0.379320</t>
+  </si>
+  <si>
+    <t>0.236087</t>
+  </si>
+  <si>
+    <t>7.120387</t>
   </si>
   <si>
     <t>涅石：本经里的明矾石 《神农本草经》卷一上经的干地黄：味甘寒，主折跌绝筋、逐血痹、填骨髓，生者尤良。
@@ -1167,19 +1287,19 @@
     <t>2026-08-17 10:01:55</t>
   </si>
   <si>
-    <t>99</t>
-  </si>
-  <si>
-    <t>0.161290</t>
-  </si>
-  <si>
-    <t>0.260417</t>
-  </si>
-  <si>
-    <t>0.385417</t>
-  </si>
-  <si>
-    <t>4.802083</t>
+    <t>100</t>
+  </si>
+  <si>
+    <t>0.159574</t>
+  </si>
+  <si>
+    <t>0.257732</t>
+  </si>
+  <si>
+    <t>0.381443</t>
+  </si>
+  <si>
+    <t>4.793814</t>
   </si>
   <si>
     <t>石钟乳：溶洞钟乳也是本草 《神农本草经》里的石钟乳：味甘温，主咳逆上气，通百节，利九窍，下乳汁。
@@ -1191,19 +1311,19 @@
     <t>2026-08-16 08:26:56</t>
   </si>
   <si>
-    <t>929</t>
-  </si>
-  <si>
-    <t>0.108137</t>
-  </si>
-  <si>
-    <t>0.287169</t>
-  </si>
-  <si>
-    <t>0.331976</t>
-  </si>
-  <si>
-    <t>5.032587</t>
+    <t>932</t>
+  </si>
+  <si>
+    <t>0.107791</t>
+  </si>
+  <si>
+    <t>0.286294</t>
+  </si>
+  <si>
+    <t>0.330964</t>
+  </si>
+  <si>
+    <t>5.026396</t>
   </si>
   <si>
     <t>玉泉：食玉之说从何而来 《神农本草经》里的玉泉（玉）：味甘平，主柔筋强骨、安魂魄、长肌肉，久服耐寒暑。
@@ -1215,19 +1335,19 @@
     <t>2026-08-15 09:43:06</t>
   </si>
   <si>
-    <t>1258</t>
-  </si>
-  <si>
-    <t>0.105863</t>
-  </si>
-  <si>
-    <t>0.241098</t>
-  </si>
-  <si>
-    <t>0.396142</t>
-  </si>
-  <si>
-    <t>5.241098</t>
+    <t>1261</t>
+  </si>
+  <si>
+    <t>0.105605</t>
+  </si>
+  <si>
+    <t>0.240563</t>
+  </si>
+  <si>
+    <t>0.396743</t>
+  </si>
+  <si>
+    <t>5.233901</t>
   </si>
   <si>
     <t>云母：六个别名的本经上品 《神农本草经》卷一石部之首的云母：味甘平，主身皮死肌、安五脏、益子精、明目。
@@ -1239,19 +1359,19 @@
     <t>2026-08-14 10:38:46</t>
   </si>
   <si>
-    <t>592</t>
-  </si>
-  <si>
-    <t>0.132042</t>
-  </si>
-  <si>
-    <t>0.270400</t>
-  </si>
-  <si>
-    <t>0.360000</t>
-  </si>
-  <si>
-    <t>4.742812</t>
+    <t>594</t>
+  </si>
+  <si>
+    <t>0.131810</t>
+  </si>
+  <si>
+    <t>0.271565</t>
+  </si>
+  <si>
+    <t>0.359425</t>
+  </si>
+  <si>
+    <t>4.748006</t>
   </si>
   <si>
     <t>丹沙：能化为汞的本经石药 《神农本草经》卷一开篇第一味药是丹沙（朱砂）：味甘微寒，养精神，安魂魄，明目。
@@ -1263,19 +1383,19 @@
     <t>2026-08-14 10:24:41</t>
   </si>
   <si>
-    <t>156</t>
-  </si>
-  <si>
-    <t>0.117647</t>
-  </si>
-  <si>
-    <t>0.251534</t>
-  </si>
-  <si>
-    <t>0.411043</t>
-  </si>
-  <si>
-    <t>5.196319</t>
+    <t>158</t>
+  </si>
+  <si>
+    <t>0.115385</t>
+  </si>
+  <si>
+    <t>0.253012</t>
+  </si>
+  <si>
+    <t>0.403614</t>
+  </si>
+  <si>
+    <t>5.210843</t>
   </si>
   <si>
     <t>黄耆：痈疽 排脓 小儿百病 《神农本草经》里的黄耆：味甘，微温，主治痈疽久败创、排脓止痛，又补虚、治小儿百病；别名戴糁，生于山谷，二月、十月采。
@@ -1286,19 +1406,19 @@
     <t>2026-08-14 10:18:02</t>
   </si>
   <si>
-    <t>636</t>
-  </si>
-  <si>
-    <t>0.103448</t>
-  </si>
-  <si>
-    <t>0.285489</t>
-  </si>
-  <si>
-    <t>0.359621</t>
-  </si>
-  <si>
-    <t>4.624606</t>
+    <t>640</t>
+  </si>
+  <si>
+    <t>0.104575</t>
+  </si>
+  <si>
+    <t>0.288854</t>
+  </si>
+  <si>
+    <t>0.357928</t>
+  </si>
+  <si>
+    <t>4.653061</t>
   </si>
   <si>
     <t>甘草：古书里写了什么？ 《神农本草经》如何记载甘草？
@@ -1310,19 +1430,19 @@
     <t>2026-08-12 10:38:33</t>
   </si>
   <si>
-    <t>807</t>
-  </si>
-  <si>
-    <t>0.210875</t>
-  </si>
-  <si>
-    <t>0.246675</t>
-  </si>
-  <si>
-    <t>0.379686</t>
-  </si>
-  <si>
-    <t>5.590085</t>
+    <t>812</t>
+  </si>
+  <si>
+    <t>0.213439</t>
+  </si>
+  <si>
+    <t>0.250301</t>
+  </si>
+  <si>
+    <t>0.377858</t>
+  </si>
+  <si>
+    <t>5.599278</t>
   </si>
 </sst>
 </file>
@@ -1689,7 +1809,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P50"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr defaultRowHeight="12.85"/>
   <cols>
     <col collapsed="false" hidden="false" max="1" min="1" style="1" width="9.5"/>
@@ -1804,195 +1924,195 @@
         <v>28</v>
       </c>
       <c r="O2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="O3" s="1" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="H4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="K4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="1" t="s">
+      <c r="H5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="K5" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="H6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="K6" s="1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>27</v>
@@ -2001,663 +2121,663 @@
         <v>27</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="H7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="L7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="O7" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="J7" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="P7" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="1" t="s">
+      <c r="H8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="J8" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="L8" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="P8" s="1" t="s">
-        <v>75</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="H9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I9" s="1" t="s">
+      <c r="L9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="J9" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="O9" s="1" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="H10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="K10" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>51</v>
-      </c>
       <c r="L10" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="H11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="J11" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>106</v>
-      </c>
       <c r="K11" s="1" t="s">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="L11" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="H12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>114</v>
-      </c>
       <c r="K12" s="1" t="s">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="N12" s="1" t="s">
         <v>39</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="H13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>121</v>
-      </c>
       <c r="K13" s="1" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="1" t="s">
+      <c r="H14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="L14" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="H15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" s="1" t="s">
+      <c r="K15" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="O15" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="J15" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="P15" s="1" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="H16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="J16" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="J16" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>83</v>
-      </c>
       <c r="L16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="H17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I17" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="J17" s="1" t="s">
-        <v>150</v>
-      </c>
       <c r="K17" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="L17" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="O17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="F18" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="J18" s="1" t="s">
-        <v>157</v>
-      </c>
       <c r="K18" s="1" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="K19" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>41</v>
-      </c>
       <c r="L19" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>75</v>
+        <v>134</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20">
@@ -2692,272 +2812,272 @@
         <v>171</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="M20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="H21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="H21" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="K21" s="1" t="s">
-        <v>180</v>
+        <v>97</v>
       </c>
       <c r="L21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N21" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="O21" s="1" t="s">
-        <v>91</v>
+        <v>134</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="H22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="K22" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="L22" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="H23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G23" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="K23" s="1" t="s">
-        <v>136</v>
+        <v>72</v>
       </c>
       <c r="L23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O23" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="M23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="P23" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="F24" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="H24" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="K24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L24" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="N24" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E25" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="H25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I25" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="L25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O25" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="L25" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="M25" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="O25" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="P25" s="1" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26">
@@ -2992,22 +3112,22 @@
         <v>215</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>26</v>
+        <v>142</v>
       </c>
       <c r="L26" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M26" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>29</v>
+        <v>126</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27">
@@ -3042,7 +3162,7 @@
         <v>222</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="L27" s="1" t="s">
         <v>27</v>
@@ -3051,13 +3171,13 @@
         <v>27</v>
       </c>
       <c r="N27" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28">
@@ -3092,22 +3212,22 @@
         <v>229</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>51</v>
+        <v>134</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M28" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N28" s="1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>28</v>
+        <v>126</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
     </row>
     <row r="29">
@@ -3142,22 +3262,22 @@
         <v>236</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="M29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N29" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>27</v>
+        <v>97</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30">
@@ -3192,22 +3312,22 @@
         <v>243</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>28</v>
+        <v>126</v>
       </c>
       <c r="O30" s="1" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
     </row>
     <row r="31">
@@ -3242,22 +3362,22 @@
         <v>250</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>74</v>
+        <v>126</v>
       </c>
       <c r="O31" s="1" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32">
@@ -3292,7 +3412,7 @@
         <v>257</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>91</v>
+        <v>39</v>
       </c>
       <c r="L32" s="1" t="s">
         <v>27</v>
@@ -3301,13 +3421,13 @@
         <v>27</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="O32" s="1" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33">
@@ -3330,19 +3450,19 @@
         <v>261</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>219</v>
+        <v>262</v>
       </c>
       <c r="H33" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="L33" s="1" t="s">
         <v>27</v>
@@ -3351,21 +3471,21 @@
         <v>27</v>
       </c>
       <c r="N33" s="1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>18</v>
@@ -3374,25 +3494,25 @@
         <v>19</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="K34" s="1" t="s">
-        <v>75</v>
+        <v>29</v>
       </c>
       <c r="L34" s="1" t="s">
         <v>27</v>
@@ -3401,10 +3521,10 @@
         <v>27</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="P34" s="1" t="s">
         <v>27</v>
@@ -3412,10 +3532,10 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>18</v>
@@ -3424,40 +3544,40 @@
         <v>19</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>23</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>278</v>
+        <v>142</v>
       </c>
       <c r="L35" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>38</v>
+        <v>71</v>
       </c>
       <c r="O35" s="1" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="36">
@@ -3492,157 +3612,157 @@
         <v>285</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>286</v>
+        <v>97</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="O36" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="P36" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="P36" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="C37" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E37" s="1" t="s">
+      <c r="F37" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I37" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="H37" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="J37" s="1" t="s">
-        <v>293</v>
-      </c>
       <c r="K37" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="L37" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N37" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="L37" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="O37" s="1" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="C38" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E38" s="1" t="s">
+      <c r="F38" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="H38" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I38" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="H38" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I38" s="1" t="s">
+      <c r="J38" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="J38" s="1" t="s">
-        <v>300</v>
-      </c>
       <c r="K38" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="C39" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E39" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="H39" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I39" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="H39" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I39" s="1" t="s">
+      <c r="J39" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="J39" s="1" t="s">
-        <v>307</v>
-      </c>
       <c r="K39" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="L39" s="1" t="s">
         <v>27</v>
@@ -3651,49 +3771,49 @@
         <v>27</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>75</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="C40" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E40" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="H40" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I40" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="H40" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="J40" s="1" t="s">
+      <c r="K40" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="K40" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="L40" s="1" t="s">
         <v>27</v>
       </c>
@@ -3701,13 +3821,13 @@
         <v>27</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>42</v>
+        <v>80</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41">
@@ -3751,13 +3871,13 @@
         <v>27</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>38</v>
+        <v>89</v>
       </c>
       <c r="O41" s="1" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="42">
@@ -3792,22 +3912,22 @@
         <v>329</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M42" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>39</v>
+        <v>97</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43">
@@ -3842,57 +3962,57 @@
         <v>336</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>337</v>
+        <v>37</v>
       </c>
       <c r="L43" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>107</v>
+        <v>39</v>
       </c>
       <c r="O43" s="1" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>75</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="C44" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="C44" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E44" s="1" t="s">
+      <c r="F44" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="G44" s="1" t="s">
+      <c r="H44" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I44" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="H44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I44" s="1" t="s">
+      <c r="J44" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="J44" s="1" t="s">
-        <v>344</v>
-      </c>
       <c r="K44" s="1" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>27</v>
@@ -3907,93 +4027,93 @@
         <v>27</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="C45" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E45" s="1" t="s">
+      <c r="F45" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="G45" s="1" t="s">
+      <c r="H45" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="H45" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="J45" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="K45" s="1" t="s">
-        <v>136</v>
+        <v>47</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="M45" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="O45" s="1" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="C46" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="C46" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E46" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="G46" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="H46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="H46" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I46" s="1" t="s">
+      <c r="J46" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="K46" s="1" t="s">
-        <v>278</v>
-      </c>
       <c r="L46" s="1" t="s">
         <v>27</v>
       </c>
@@ -4001,13 +4121,13 @@
         <v>27</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47">
@@ -4042,7 +4162,7 @@
         <v>365</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="L47" s="1" t="s">
         <v>27</v>
@@ -4051,13 +4171,13 @@
         <v>27</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -4092,22 +4212,22 @@
         <v>372</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="L48" s="1" t="s">
         <v>27</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49">
@@ -4142,7 +4262,7 @@
         <v>379</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L49" s="1" t="s">
         <v>27</v>
@@ -4151,13 +4271,13 @@
         <v>27</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>74</v>
+        <v>27</v>
       </c>
       <c r="O49" s="1" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="50">
@@ -4192,22 +4312,272 @@
         <v>386</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>91</v>
+        <v>208</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M50" s="1" t="s">
         <v>27</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="P50" s="1" t="s">
-        <v>39</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M51" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N51" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="O51" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="P51" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N52" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O52" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="P52" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L53" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M53" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="N53" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O53" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P53" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="J54" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="L54" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M54" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N54" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O54" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P54" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N55" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O55" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P55" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>